<commit_message>
feat: add visual-layout sorting rule (§4-a) and regenerate both Excels
Skill change:
- Add §4-a: 用例排序规则 (visual layout priority)
  - Core principle: top→bottom, left→right matching page layout
  - Sort algorithm: page-level → area position → sub-position
  - Example sort map for 托工订单 list page
  - Reusable Python sort_key template

Excel regeneration:
- List page (56 cases): 筛选区查询 → 工具栏按钮(新增→导出→打印→料件预计领用→流程设置) → VTable交互 → 边界/异常 → 页面级
- New page (35 cases): 基本信息 → 货物信息(商品库) → 附件 → 校验/提交 → 页面导航

Same-function cases now grouped together for linear test execution
</commit_message>
<xml_diff>
--- a/测试用例_托工管理_托工订单新增_2026-06-22.xlsx
+++ b/测试用例_托工管理_托工订单新增_2026-06-22.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="字段矩阵" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="测试数据" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -759,22 +759,22 @@
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A003</t>
+          <t>NB_TGDD_A011</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>新增—选择供应商后供应商编码自动填充</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>新增—必填字段为空时标红星提示</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>验证供应商名称下拉选择后编码字段自动带出</t>
+          <t>验证必填字段左侧有红色星号标识</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -805,20 +805,19 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>1. 点击供应商名称下拉框
-2. 选择「企业名称11」
-3. 观察供应商编码字段变化</t>
+          <t>1. 进入新增页
+2. 观察基本信息区域各字段左侧标识</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>供应商名称:企业名称11
-预期编码:供应商编码0011</t>
+          <t>操作:观察字段标注</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>供应商编码自动填充为「供应商编码0011」</t>
+          <t>必填字段（供应商/编码/计税类别/托运责任/负责人/交付地点/进货仓库/订单类型/币别）左侧有红色星号
+非必填字段（托工单号/邮箱/备注）无星号</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -835,22 +834,22 @@
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A004</t>
+          <t>NB_TGDD_A003</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>新增—切换供应商后供应商编码同步更新</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—选择供应商后供应商编码自动填充</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>验证切换不同供应商时编码正确更新</t>
+          <t>验证供应商名称下拉选择后编码字段自动带出</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -876,26 +875,25 @@
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 已选择供应商「企业名称11」</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>1. 重新点击供应商名称下拉
-2. 切换为「中山原材料供应商」
-3. 观察编码变化</t>
+          <t>1. 点击供应商名称下拉框
+2. 选择「企业名称11」
+3. 观察供应商编码字段变化</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>切换前:企业名称11→供应商编码0011
-切换后:中山原材料供应商</t>
+          <t>供应商名称:企业名称11
+预期编码:供应商编码0011</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>供应商编码更新为中山原材料供应商对应编码
-不保留旧编码</t>
+          <t>供应商编码自动填充为「供应商编码0011」</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -912,22 +910,22 @@
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A005</t>
+          <t>NB_TGDD_A004</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>新增—进货仓库下拉16个选项完整可选</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>新增—切换供应商后供应商编码同步更新</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>验证进货仓库下拉全部16个选项可正常展示和选择</t>
+          <t>验证切换不同供应商时编码正确更新</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -953,27 +951,26 @@
       <c r="I6" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 已选择供应商「企业名称11」</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>1. 点击进货仓库下拉框
-2. 滚动查看全部选项
-3. 选择「成品仓」</t>
+          <t>1. 重新点击供应商名称下拉
+2. 切换为「中山原材料供应商」
+3. 观察编码变化</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>字段:进货仓库
-选项数:16
-选择:成品仓</t>
+          <t>切换前:企业名称11→供应商编码0011
+切换后:中山原材料供应商</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>下拉展开显示16个仓库
-选择「成品仓」后字段值更新</t>
+          <t>供应商编码更新为对应编码
+不保留旧编码</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr"/>
@@ -990,12 +987,12 @@
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A006</t>
+          <t>NB_TGDD_A005</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>新增—计税类别切换（不计税/应税内含/应税外加）</t>
+          <t>新增—进货仓库下拉16个选项完整可选</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1005,7 +1002,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>验证计税类别3个选项切换正常且可能影响金额展示</t>
+          <t>验证进货仓库下拉全部16个选项可正常展示和选择</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1036,21 +1033,22 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>1. 点击计税类别下拉
-2. 依次切换「不计税」「应税内含」「应税外加」
-3. 观察字段变化</t>
+          <t>1. 点击进货仓库下拉框
+2. 滚动查看全部选项
+3. 选择「成品仓」</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>字段:计税类别
-选项:不计税/应税内含/应税外加</t>
+          <t>字段:进货仓库
+选项数:16
+选择:成品仓</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>3个选项均可选中
-应税内含/外加切换后金额相关字段可能变化</t>
+          <t>下拉展开显示16个仓库
+选择「成品仓」后字段值更新</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
@@ -1067,22 +1065,22 @@
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A007</t>
+          <t>NB_TGDD_A006</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>新增—托运责任仅限2个选项（新增页受限子集）</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—计税类别切换（不计税/应税内含/应税外加）</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>验证新增页托运责任下拉仅显示2个选项（与列表筛选的8个不同）</t>
+          <t>验证计税类别3个选项切换正常且可能影响金额展示</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1113,21 +1111,20 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>1. 点击托运责任下拉
-2. 记录全部选项</t>
+          <t>1. 点击计税类别下拉
+2. 依次切换「不计税」「应税内含」「应税外加」</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>字段:托运责任
-选项数:2
-选项:供应商送货/我司提货</t>
+          <t>字段:计税类别
+选项:不计税/应税内含/应税外加</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>仅显示2个选项
-确认与列表页筛选的8个选项不同（为业务受限子集）</t>
+          <t>3个选项均可选中
+应税内含/外加切换后金额相关字段可能变化</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
@@ -1144,22 +1141,22 @@
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A008</t>
+          <t>NB_TGDD_A007</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>新增—交付地点下拉选择</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>新增—托运责任仅限2个选项（新增页受限子集）</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>验证交付地点下拉选项可选择</t>
+          <t>验证新增页托运责任下拉仅显示2个选项</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1190,20 +1187,21 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>1. 点击交付地点下拉
-2. 选择「中山世通医疗」</t>
+          <t>1. 点击托运责任下拉
+2. 记录全部选项</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>字段:交付地点
-选项:中山/中山世通医疗
-选择:中山世通医疗</t>
+          <t>字段:托运责任
+选项数:2
+选项:供应商送货/我司提货</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>交付地点字段值更新为「中山世通医疗」</t>
+          <t>仅显示2个选项
+确认为业务受限子集</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
@@ -1220,22 +1218,22 @@
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A009</t>
+          <t>NB_TGDD_A008</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>新增—订单币别下拉22种货币可选</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—交付地点下拉选择</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>验证订单币别下拉包含完整货币列表</t>
+          <t>验证交付地点下拉选项可选择</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1266,22 +1264,19 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>1. 点击订单币别下拉
-2. 查看选项
-3. 选择「美元」</t>
+          <t>1. 点击交付地点下拉
+2. 选择「中山世通医疗」</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>字段:订单币别
-默认:人民币
-切换为:美元</t>
+          <t>字段:交付地点
+选项:中山/中山世通医疗</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>下拉包含22种货币
-选择「美元」后字段更新</t>
+          <t>交付地点字段值更新为「中山世通医疗」</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
@@ -1298,22 +1293,22 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A010</t>
+          <t>NB_TGDD_A009</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>新增—未关联货物信息时提交提示</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>新增—订单币别下拉22种货币可选</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>验证未添加货物时点击生成给出明确提示</t>
+          <t>验证订单币别下拉包含完整货币列表</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1339,28 +1334,27 @@
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入新增页
-3. 已填写基本信息（供应商等）
-4. 货物信息为空</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>1. 填写基本信息
-2. 货物信息区域保持空
-3. 点击「生成托工订单」</t>
+          <t>1. 点击订单币别下拉
+2. 查看选项
+3. 选择「美元」</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>基本信息:已填
-货物信息:（空）</t>
+          <t>字段:订单币别
+默认:人民币
+切换为:美元</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>弹出提示「采购订单未关联货物信息！」
-不提交请求</t>
+          <t>下拉包含22种货币
+选择「美元」后字段更新</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr"/>
@@ -1377,12 +1371,12 @@
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A011</t>
+          <t>NB_TGDD_A012</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>新增—必填字段为空时标红星提示</t>
+          <t>新增—托工单号为非必填可留空</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1392,7 +1386,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>验证必填字段左侧有红色星号标识</t>
+          <t>验证托工单号字段留空不阻塞提交</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1418,24 +1412,27 @@
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 进入新增页</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>1. 进入新增页
-2. 观察基本信息区域各字段左侧标识</t>
+          <t>1. 填写必填字段
+2. 托工单号留空
+3. 添加货物后点击生成</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>操作:观察字段标注</t>
+          <t>托工单号:（空）
+其他必填:已填
+货物:已添加</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>供应商名称/供应商编码/计税类别/托运责任/托工负责人/交付地点/进货仓库/订单类型/订单币别左侧有红色星号
-非必填字段（托工单号/邮箱/备注）无星号</t>
+          <t>提交成功
+系统自动生成托工单号</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
@@ -1452,12 +1449,12 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A012</t>
+          <t>NB_TGDD_A013</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>新增—托工单号为非必填可留空</t>
+          <t>新增—接收提醒邮箱格式校验</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1467,7 +1464,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>验证托工单号字段留空不阻塞提交（由系统自动生成）</t>
+          <t>验证邮箱字段填写非法格式时的提示</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1493,27 +1490,23 @@
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入新增页</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>1. 填写必填字段
-2. 托工单号留空
-3. 添加货物后点击生成</t>
+          <t>1. 在接收提醒邮箱输入「not-an-email」
+2. 尝试提交</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>托工单号:（空）
-其他必填:已填
-货物:已添加</t>
+          <t>接收提醒邮箱:not-an-email</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>提交成功
-系统自动生成托工单号</t>
+          <t>系统应提示邮箱格式不正确或接受但给出警告</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr"/>
@@ -1530,12 +1523,12 @@
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A013</t>
+          <t>NB_TGDD_G009</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>新增—接收提醒邮箱格式校验</t>
+          <t>货物—用料清单表格展示</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1545,7 +1538,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>验证邮箱字段填写非法格式时的提示</t>
+          <t>验证用料清单子表包含正确的列定义</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1560,7 +1553,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>异常测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1576,19 +1569,18 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>1. 在接收提醒邮箱输入「not-an-email」
-2. 尝试提交</t>
+          <t>1. 观察货物信息区域的用料清单子表
+2. 记录表头列</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>接收提醒邮箱:not-an-email</t>
+          <t>操作:查看用料清单表头</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>系统应提示邮箱格式不正确
-或接受但给出警告</t>
+          <t>用料清单表包含:项/物料编码/应发料数量/成品编码/物料名称/物料型号/单位/实发数量/待发数量/操作</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
@@ -1605,12 +1597,12 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A014</t>
+          <t>NB_TGDD_G001</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>新增—点击返回按钮回到列表页</t>
+          <t>货物—从商品库选择按钮打开弹窗</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1620,7 +1612,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>验证返回按钮可正常回到列表页且关闭新增Tab</t>
+          <t>验证点击从商品库选择弹出商品库弹窗</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1646,25 +1638,25 @@
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页
-3. 未填写数据</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>1. 点击「返回」按钮
-2. 观察页面变化</t>
+          <t>1. 滚动到货物信息区域
+2. 点击「从商品库选择」按钮</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>操作:返回</t>
+          <t>操作:从商品库选择</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>新增Tab关闭
-回到托工订单列表页</t>
+          <t>弹出商品库弹窗
+标题为「商品库」
+包含34列VTable和筛选区</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
@@ -1681,22 +1673,22 @@
     <row r="16" ht="80" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_A015</t>
+          <t>NB_TGDD_G002</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>新增—点击列表按钮回到列表页</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>货物—商品库弹窗按货物状态和商品类型筛选</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>验证列表按钮功能与返回一致</t>
+          <t>验证商品库弹窗内筛选功能正常</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1722,23 +1714,27 @@
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 商品库弹窗已打开
+3. VTable数据已加载</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>1. 点击「列表」按钮
-2. 观察页面变化</t>
+          <t>1. 在弹窗筛选区选择货物状态
+2. 选择商品类型
+3. 等待列表刷新
+4. 勾选商品行</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>操作:列表</t>
+          <t>筛选:货物状态+商品类型</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>回到托工订单列表页</t>
+          <t>列表按筛选条件过滤
+可勾选筛选后的商品行</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
@@ -1755,22 +1751,22 @@
     <row r="17" ht="80" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G001</t>
+          <t>NB_TGDD_G005</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>货物—从商品库选择按钮打开弹窗</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>货物—商品库弹窗重置筛选条件</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>验证点击从商品库选择弹出商品库弹窗</t>
+          <t>验证弹窗内重置按钮恢复全部商品列表</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1796,25 +1792,26 @@
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 商品库弹窗已打开
+3. 已设置筛选条件</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>1. 滚动到货物信息区域
-2. 点击「从商品库选择」按钮</t>
+          <t>1. 设置货物状态筛选
+2. 点击「重置」按钮
+3. 观察列表变化</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>操作:从商品库选择</t>
+          <t>操作:重置</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>弹出商品库弹窗
-标题为「商品库」
-包含34列VTable和筛选区</t>
+          <t>筛选条件清空
+列表恢复显示全部商品</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
@@ -1831,22 +1828,22 @@
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G002</t>
+          <t>NB_TGDD_G006</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>货物—商品库弹窗按货物状态和商品类型筛选</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>货物—商品库VTable复选框全选</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>验证商品库弹窗内筛选功能正常</t>
+          <t>验证商品库VTable表头复选框全选功能</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1878,21 +1875,20 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>1. 在弹窗筛选区选择货物状态
-2. 选择商品类型
-3. 等待列表刷新
-4. 勾选商品行</t>
+          <t>1. 点击商品库VTable表头复选框
+2. 观察所有行勾选状态
+3. 再次点击取消全选</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>筛选:货物状态+商品类型</t>
+          <t>操作:全选→取消全选</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>列表按筛选条件过滤
-可勾选筛选后的商品行</t>
+          <t>全选时所有商品行被勾选
+取消时全部取消</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
@@ -1987,12 +1983,12 @@
     <row r="20" ht="80" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G004</t>
+          <t>NB_TGDD_G007</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>货物—商品库弹窗关闭不添加</t>
+          <t>货物—添加多个商品</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2002,7 +1998,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>验证点击关闭按钮不添加任何商品</t>
+          <t>验证一次添加多个商品到货物信息表</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2028,25 +2024,24 @@
       <c r="I20" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 商品库弹窗已打开
-3. 已勾选商品</t>
+2. 商品库弹窗已打开</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>1. 勾选商品行
-2. 点击「关闭」按钮</t>
+          <t>1. 勾选3个商品行
+2. 点击「添加」</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>操作:关闭</t>
+          <t>勾选商品数:3
+操作:添加</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>弹窗关闭
-货物信息表中无新增商品</t>
+          <t>货物信息委外商品表中出现3行商品数据</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
@@ -2063,12 +2058,12 @@
     <row r="21" ht="80" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G005</t>
+          <t>NB_TGDD_G004</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>货物—商品库弹窗重置筛选条件</t>
+          <t>货物—商品库弹窗关闭不添加</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2078,7 +2073,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>验证弹窗内重置按钮恢复全部商品列表</t>
+          <t>验证点击关闭按钮不添加任何商品</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2105,25 +2100,24 @@
         <is>
           <t>1. 已登录SCM系统
 2. 商品库弹窗已打开
-3. 已设置筛选条件</t>
+3. 已勾选商品</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>1. 设置货物状态筛选
-2. 点击「重置」按钮
-3. 观察列表变化</t>
+          <t>1. 勾选商品行
+2. 点击「关闭」按钮</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>操作:重置</t>
+          <t>操作:关闭</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>筛选条件清空
-列表恢复显示全部商品</t>
+          <t>弹窗关闭
+货物信息表中无新增商品</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr"/>
@@ -2140,12 +2134,12 @@
     <row r="22" ht="80" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G006</t>
+          <t>NB_TGDD_G008</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>货物—商品库VTable复选框全选</t>
+          <t>货物—委外商品表中删除商品行</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -2155,7 +2149,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>验证商品库VTable表头复选框全选功能</t>
+          <t>验证已添加的商品行可删除</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2181,26 +2175,23 @@
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 商品库弹窗已打开
-3. VTable数据已加载</t>
+2. 货物信息中已有至少1个商品</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>1. 点击商品库VTable表头复选框
-2. 观察所有行勾选状态
-3. 再次点击取消全选</t>
+          <t>1. 在委外商品表中找到某行的操作列
+2. 点击删除按钮</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>操作:全选→取消全选</t>
+          <t>操作:删除商品行</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>全选时所有商品行被勾选
-取消时全部取消</t>
+          <t>该商品行从货物信息表中移除</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
@@ -2217,12 +2208,12 @@
     <row r="23" ht="80" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G007</t>
+          <t>NB_TGDD_G010</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>货物—添加多个商品</t>
+          <t>货物—委外商品表中需交付日期为日期选择器</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -2232,7 +2223,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>验证一次添加多个商品到货物信息表</t>
+          <t>验证商品添加后需交付日期列支持日期选择</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2258,25 +2249,26 @@
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 商品库弹窗已打开</t>
+2. 货物信息中已有商品</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>1. 勾选3个商品行
-2. 点击「添加」</t>
+          <t>1. 在委外商品表中找到需交付日期列
+2. 点击触发日期选择器
+3. 选择日期</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>勾选商品数:3
-操作:添加</t>
+          <t>字段:需交付日期
+操作:日期选择</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>货物信息委外商品表中出现3行商品数据
-每行包含商品名称/识别码/型号等字段</t>
+          <t>日期选择器弹出
+可选择日期并回填到单元格</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
@@ -2293,22 +2285,22 @@
     <row r="24" ht="80" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G008</t>
+          <t>NB_TGDD_U001</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>货物—委外商品表中删除商品行</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>附件—点击上传区域触发文件选择</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>验证已添加的商品行可删除</t>
+          <t>验证点击上传区域能触发浏览器文件选择对话框</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2328,30 +2320,29 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 货物信息中已有至少1个商品</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>1. 在委外商品表中找到某行的操作列
-2. 点击删除按钮
-3. 确认删除</t>
+          <t>1. 滚动到附件列表区域
+2. 点击上传区域</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>操作:删除商品行</t>
+          <t>操作:点击上传</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>该商品行从货物信息表中移除</t>
+          <t>触发浏览器文件选择对话框</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
@@ -2368,22 +2359,22 @@
     <row r="25" ht="80" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G009</t>
+          <t>NB_TGDD_U002</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>货物—用料清单表格展示</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>附件—上传PDF文件成功并显示在列表</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>验证用料清单子表包含正确的列定义</t>
+          <t>验证上传有效PDF文件后列表中出现记录</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2403,29 +2394,32 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 准备一个≤5MB的PDF文件</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>1. 观察货物信息区域的用料清单子表
-2. 记录表头列</t>
+          <t>1. 点击上传区域
+2. 选择PDF文件
+3. 等待上传完成</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>操作:查看用料清单表头</t>
+          <t>文件类型:pdf
+文件大小:≤5MB</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>用料清单表包含:项/物料编码/应发料数量/成品编码/成名名称/物料名称/物料型号/单位/实发数量/待发数量/操作</t>
+          <t>附件列表中新增一行
+显示文件名/文件大小/上传时间</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
@@ -2442,12 +2436,12 @@
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_G010</t>
+          <t>NB_TGDD_U007</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>货物—委外商品表中需交付日期为日期选择器</t>
+          <t>附件—上传多个不同格式文件</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -2457,7 +2451,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>验证商品添加后需交付日期列支持日期选择</t>
+          <t>验证同时上传PDF/PNG/XLSX三种格式</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2477,32 +2471,31 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 货物信息中已有商品</t>
+2. 准备PDF/PNG/XLSX各一个</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>1. 在委外商品表中找到需交付日期列
-2. 点击触发日期选择器
-3. 选择日期</t>
+          <t>1. 依次上传PDF、PNG、XLSX文件
+2. 观察列表</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>字段:需交付日期
-操作:日期选择</t>
+          <t>文件数:3
+格式:pdf/png/xlsx</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>日期选择器弹出
-可选择日期并回填到单元格</t>
+          <t>3个文件全部上传成功
+列表中显示3行记录</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr"/>
@@ -2519,22 +2512,22 @@
     <row r="27" ht="80" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U001</t>
+          <t>NB_TGDD_U006</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>附件—点击上传区域触发文件选择</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>附件—删除已上传的附件</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>验证点击上传区域能触发浏览器文件选择对话框</t>
+          <t>验证附件列表中的删除操作</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2560,23 +2553,23 @@
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 进入托工订单新增页</t>
+2. 附件列表中已有至少1个文件</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>1. 滚动到附件列表区域
-2. 点击上传区域</t>
+          <t>1. 在附件列表中找到某行的操作列
+2. 点击删除按钮</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>操作:点击上传</t>
+          <t>操作:删除附件</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>触发浏览器文件选择对话框</t>
+          <t>该附件从列表中移除</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
@@ -2593,22 +2586,22 @@
     <row r="28" ht="80" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U002</t>
+          <t>NB_TGDD_U003</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>附件—上传PDF文件成功并显示在列表</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>附件—上传超过5个文件时提示限制</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>验证上传有效PDF文件后列表中出现记录</t>
+          <t>验证上传第6个文件时系统给出限制提示</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2634,26 +2627,25 @@
       <c r="I28" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 准备一个≤5MB的PDF文件</t>
+2. 已上传5个文件</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>1. 点击上传区域
-2. 选择PDF文件
-3. 等待上传完成</t>
+          <t>1. 尝试上传第6个文件
+2. 观察系统反应</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>文件类型:pdf
-文件大小:≤5MB</t>
+          <t>已上传:5个
+第6个:任意文件</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>附件列表中新增一行
-显示文件名/文件大小/上传时间</t>
+          <t>系统提示「最大可批量上传5个文件」
+第6个文件不被接受</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
@@ -2670,12 +2662,12 @@
     <row r="29" ht="80" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U003</t>
+          <t>NB_TGDD_U004</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>附件—上传超过5个文件时提示限制</t>
+          <t>附件—上传超过5MB文件时提示限制</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2685,7 +2677,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>验证上传第6个文件时系统给出限制提示</t>
+          <t>验证上传超5MB文件时系统给出提示</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2700,7 +2692,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>边界值测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2711,25 +2703,23 @@
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 已上传5个文件</t>
+2. 准备一个&gt;5MB的文件</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>1. 尝试上传第6个文件
+          <t>1. 尝试上传&gt;5MB的文件
 2. 观察系统反应</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>已上传:5个
-第6个:任意文件</t>
+          <t>文件大小:&gt;5MB</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>系统提示「最大可批量上传5个文件」
-第6个文件不被接受</t>
+          <t>系统提示「每个文件不超过5MB」</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr"/>
@@ -2746,12 +2736,12 @@
     <row r="30" ht="80" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U004</t>
+          <t>NB_TGDD_U005</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>附件—上传超过5MB文件时提示限制</t>
+          <t>附件—上传不支持的文件格式</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2761,7 +2751,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>验证上传超5MB文件时系统给出提示</t>
+          <t>验证上传不支持格式时系统提示</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2776,7 +2766,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>边界值测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2787,23 +2777,23 @@
       <c r="I30" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 准备一个&gt;5MB的文件</t>
+2. 准备一个.exe文件</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>1. 尝试上传&gt;5MB的文件
+          <t>1. 尝试上传.exe文件
 2. 观察系统反应</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>文件大小:&gt;5MB</t>
+          <t>文件类型:exe</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>系统提示「每个文件不超过5MB」</t>
+          <t>系统提示不支持该格式或不显示在文件选择器中</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr"/>
@@ -2820,22 +2810,22 @@
     <row r="31" ht="80" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U005</t>
+          <t>NB_TGDD_A010</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>附件—上传不支持的文件格式</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—未关联货物信息时提交提示</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>验证上传不支持格式时系统提示</t>
+          <t>验证未添加货物时点击生成给出明确提示</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2850,35 +2840,39 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>异常测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>附件</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 准备一个.exe文件</t>
+2. 进入新增页
+3. 已填写基本信息
+4. 货物信息为空</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>1. 尝试上传.exe文件
-2. 观察系统反应</t>
+          <t>1. 填写基本信息
+2. 货物信息区域保持空
+3. 点击「生成托工订单」</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>文件类型:exe</t>
+          <t>基本信息:已填
+货物信息:（空）</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>系统提示不支持该格式
-或不显示在文件选择器中</t>
+          <t>弹出提示「采购订单未关联货物信息！」
+不提交请求</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -2895,22 +2889,22 @@
     <row r="32" ht="80" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U006</t>
+          <t>NB_TGDD_S002</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>附件—删除已上传的附件</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—无附件提交（附件为非必填）</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>验证附件列表中的删除操作</t>
+          <t>验证不传附件也能成功提交</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2930,29 +2924,33 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>附件</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 附件列表中已有至少1个文件</t>
+2. 填写基本信息+选择商品
+3. 不上传附件</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>1. 在附件列表中找到某行的操作列
-2. 点击删除按钮</t>
+          <t>1. 填写必填字段+添加商品
+2. 附件保持空
+3. 点击「生成托工订单」</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>操作:删除附件</t>
+          <t>附件:（无）
+其他:已填</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>该附件从列表中移除</t>
+          <t>提交成功
+附件为空不影响订单创建</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr"/>
@@ -2969,22 +2967,22 @@
     <row r="33" ht="80" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_U007</t>
+          <t>NB_TGDD_S001</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>附件—上传多个不同格式文件</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>新增—完整流程：填写基本信息+选择商品+上传附件+提交</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>验证同时上传PDF/PNG/XLSX三种格式</t>
+          <t>验证端到端新增托工订单全流程</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3004,93 +3002,17 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>附件</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>1. 已登录SCM系统
-2. 准备PDF/PNG/XLSX各一个</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>1. 依次上传PDF、PNG、XLSX文件
-2. 观察列表</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>文件数:3
-格式:pdf/png/xlsx</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="inlineStr">
-        <is>
-          <t>3个文件全部上传成功
-列表中显示3行记录</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>Hooplus1ce</t>
-        </is>
-      </c>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="80" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>NB_TGDD_S001</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>新增—完整流程：填写基本信息+选择商品+上传附件+提交</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>验证端到端新增托工订单全流程</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>托工管理</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>托工订单新增</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>新增</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
 2. 供应商、商品数据就绪
 3. 准备1个PDF附件</t>
         </is>
       </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>1. 进入新增页
 2. 选择供应商「企业名称11」→编码自动填充
@@ -3101,7 +3023,7 @@
 7. 点击「生成托工订单」</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>供应商:企业名称11
 进货仓库:成品仓
@@ -3110,7 +3032,7 @@
 附件:1个PDF</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>提交成功
 弹出成功提示
@@ -3118,6 +3040,82 @@
 列表页刷新后可见新订单</t>
         </is>
       </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="80" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A014</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>新增—点击返回按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>验证返回按钮可正常回到列表页且关闭新增Tab</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>托工订单新增</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入托工订单新增页
+3. 未填写数据</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>1. 点击「返回」按钮
+2. 观察页面变化</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>操作:返回</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>新增Tab关闭
+回到托工订单列表页</t>
+        </is>
+      </c>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
@@ -3132,22 +3130,22 @@
     <row r="35" ht="80" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NB_TGDD_S002</t>
+          <t>NB_TGDD_A015</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>新增—无附件提交（附件为非必填）</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>新增—点击列表按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>验证不传附件也能成功提交</t>
+          <t>验证列表按钮功能与返回一致</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3173,27 +3171,23 @@
       <c r="I35" s="3" t="inlineStr">
         <is>
           <t>1. 已登录SCM系统
-2. 填写基本信息+选择商品
-3. 不上传附件</t>
+2. 进入托工订单新增页</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>1. 填写必填字段+添加商品
-2. 附件保持空
-3. 点击「生成托工订单」</t>
+          <t>1. 点击「列表」按钮
+2. 观察页面变化</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>附件:（无）
-其他:已填</t>
+          <t>操作:列表</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>提交成功
-附件为空不影响订单创建</t>
+          <t>回到托工订单列表页</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
@@ -3269,9 +3263,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>切换回新增页后之前填写的数据保持
-供应商选择不变
-托工负责人值不变</t>
+          <t>切换回新增页后之前填写的数据保持</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr"/>
@@ -3296,814 +3288,1195 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>区域</t>
+          <t>用例编号</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>字段/按钮</t>
+          <t>用例标题</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>字段/操作</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>默认值/选项</t>
+          <t>测试输入值</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>联动行为</t>
+          <t>预期</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>供应商名称</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>新增—从列表页点击新增按钮进入新增页</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>从列表页点击新增按钮进入新增页</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>8个供应商</t>
+          <t>操作:点击新增</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>选择后→供应商编码自动填充</t>
+          <t>P0</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>供应商编码</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown+text</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>新增—页面加载时字段默认值校验</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>页面加载时字段默认值校验</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>8个编码</t>
+          <t>字段默认值:
+托运责任=供应商送货
+订单类型=委外加工
+订单币别=人民币
+托工负责人=NB_Hoo
+接收提醒邮箱=Hoo</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>随供应商名称联动</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>计税类别</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A011</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>新增—必填字段为空时标红星提示</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>必填字段为空时标红星提示</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>不计税/应税内含/应税外加</t>
+          <t>操作:观察字段标注</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>托运责任</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A003</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>新增—选择供应商后供应商编码自动填充</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>选择供应商后供应商编码自动填充</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>供应商送货(默认)/我司提货</t>
+          <t>供应商名称:企业名称11
+预期编码:供应商编码0011</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>托工负责人</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A004</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>新增—切换供应商后供应商编码同步更新</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>切换供应商后供应商编码同步更新</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>NB_Hoo(当前用户)</t>
+          <t>切换前:企业名称11→供应商编码0011
+切换后:中山原材料供应商</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>交付地点</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A005</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>新增—进货仓库下拉16个选项完整可选</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>进货仓库下拉16个选项完整可选</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>中山/中山世通医疗</t>
+          <t>字段:进货仓库
+选项数:16
+选择:成品仓</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>进货仓库</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A006</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>新增—计税类别切换（不计税/应税内含/应税外加）</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>计税类别切换（不计税/应税内含/应税外加）</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>16个仓库</t>
+          <t>字段:计税类别
+选项:不计税/应税内含/应税外加</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>订单类型</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A007</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>新增—托运责任仅限2个选项（新增页受限子集）</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>托运责任仅限2个选项（新增页受限子集）</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>委外加工(默认)/普通采购</t>
+          <t>字段:托运责任
+选项数:2
+选项:供应商送货/我司提货</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>订单币别</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A008</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>新增—交付地点下拉选择</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>交付地点下拉选择</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>人民币(默认)+21种</t>
+          <t>字段:交付地点
+选项:中山/中山世通医疗</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>托工单号</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A009</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>新增—订单币别下拉22种货币可选</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>订单币别下拉22种货币可选</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>(留空,系统自动生成)</t>
+          <t>字段:订单币别
+默认:人民币
+切换为:美元</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>接收提醒邮箱</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A012</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>新增—托工单号为非必填可留空</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>托工单号为非必填可留空</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Hooplus1ce@hoolinks.com</t>
+          <t>托工单号:（空）
+其他必填:已填
+货物:已添加</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>基本信息</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A013</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>新增—接收提醒邮箱格式校验</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>接收提醒邮箱格式校验</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>(空)</t>
+          <t>接收提醒邮箱:not-an-email</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>货物信息</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>从商品库选择</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>button_modal</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G009</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>货物—用料清单表格展示</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>用料清单表格展示</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>打开商品库弹窗</t>
+          <t>操作:查看用料清单表头</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>弹窗含34列VTable+2个筛选字段</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>货物信息→商品库</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>货物状态</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown(弹窗内)</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G001</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>货物—从商品库选择按钮打开弹窗</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>从商品库选择按钮打开弹窗</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>筛选字段</t>
+          <t>操作:从商品库选择</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>货物信息→商品库</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>商品类型</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>select_dropdown(弹窗内)</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G002</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>货物—商品库弹窗按货物状态和商品类型筛选</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>商品库弹窗按货物状态和商品类型筛选</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>筛选字段</t>
+          <t>筛选:货物状态+商品类型</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>货物信息→商品库</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>VTable复选框</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>checkbox(弹窗内)</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G005</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>货物—商品库弹窗重置筛选条件</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>商品库弹窗重置筛选条件</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>勾选商品行</t>
+          <t>操作:重置</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>货物信息→商品库</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>添加/关闭/重置</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>button(弹窗内)</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G006</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>货物—商品库VTable复选框全选</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>商品库VTable复选框全选</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>确认添加或取消</t>
+          <t>操作:全选→取消全选</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>添加→回填商品;关闭→不添加</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>货物信息</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>委外商品表(16列)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>table</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G003</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>货物—勾选商品后点击添加回填到订单</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>勾选商品后点击添加回填到订单</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>项/单价/金额/配方号/商品名称/识别码/型号/包装方式/单位1/单位2/需交付日期/已进货数量/已退货数量/操作</t>
+          <t>勾选商品数:1
+操作:添加</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>从商品库添加后自动填充</t>
+          <t>P0</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>货物信息</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>用料清单表(12列)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>table</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G007</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>货物—添加多个商品</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>添加多个商品</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>项/物料编码/应发料数量/成品编码/物料名称/物料型号/单位/实发数量/待发数量/操作</t>
+          <t>勾选商品数:3
+操作:添加</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>商品确定后自动计算</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>附件列表</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>文件上传区域</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>file_upload</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G004</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>货物—商品库弹窗关闭不添加</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>商品库弹窗关闭不添加</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>拖拽或点击</t>
+          <t>操作:关闭</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>最多5个文件,每个≤5MB,14种格式</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>附件列表</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>附件表格</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>table</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G008</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>货物—委外商品表中删除商品行</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>委外商品表中删除商品行</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>序号/文件名称/文件大小/上传时间/操作</t>
+          <t>操作:删除商品行</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>上传后自动填充</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>页面按钮</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>返回</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>button_nav</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_G010</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>货物—委外商品表中需交付日期为日期选择器</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>委外商品表中需交付日期为日期选择器</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>关闭新增Tab→列表页</t>
+          <t>字段:需交付日期
+操作:日期选择</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>页面按钮</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>列表</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>button_nav</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U001</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>附件—点击上传区域触发文件选择</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>点击上传区域触发文件选择</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>关闭新增Tab→列表页</t>
+          <t>操作:点击上传</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>页面按钮</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>生成托工订单</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>button_submit</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U002</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>附件—上传PDF文件成功并显示在列表</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>上传PDF文件成功并显示在列表</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>提交创建</t>
+          <t>文件类型:pdf
+文件大小:≤5MB</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>校验:必须关联货物信息</t>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U007</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>附件—上传多个不同格式文件</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>上传多个不同格式文件</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>附件</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>文件数:3
+格式:pdf/png/xlsx</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U006</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>附件—删除已上传的附件</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>删除已上传的附件</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>附件</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>操作:删除附件</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U003</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>附件—上传超过5个文件时提示限制</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>上传超过5个文件时提示限制</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>附件</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>已上传:5个
+第6个:任意文件</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U004</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>附件—上传超过5MB文件时提示限制</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>上传超过5MB文件时提示限制</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>附件</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>文件大小:&gt;5MB</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_U005</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>附件—上传不支持的文件格式</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>上传不支持的文件格式</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>附件</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>文件类型:exe</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A010</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>新增—未关联货物信息时提交提示</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>未关联货物信息时提交提示</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>基本信息:已填
+货物信息:（空）</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_S002</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>新增—无附件提交（附件为非必填）</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>无附件提交（附件为非必填）</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>附件:（无）
+其他:已填</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_S001</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>新增—完整流程：填写基本信息+选择商品+上传附件+提交</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>完整流程：填写基本信息+选择商品+上传附件+提交</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>供应商:企业名称11
+进货仓库:成品仓
+交付地点:中山世通医疗
+商品:1个
+附件:1个PDF</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A014</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>新增—点击返回按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>点击返回按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>操作:返回</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A015</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>新增—点击列表按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>点击列表按钮回到列表页</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>操作:列表</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_S003</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>新增—已填写表单切换Tab再切回数据保持</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>已填写表单切换Tab再切回数据保持</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>操作:Tab切换</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
     </row>

</xml_diff>